<commit_message>
Update Polymarket 30-day dashboard data
</commit_message>
<xml_diff>
--- a/docs/data/kalshi_cumulative_topic_share.xlsx
+++ b/docs/data/kalshi_cumulative_topic_share.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -488,19 +488,19 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>185100.03</v>
+        <v>338131.31</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>71.21069433</v>
+        <v>83.15975802</v>
       </c>
       <c r="E2" t="n">
-        <v>205</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -509,97 +509,118 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>50871.54</v>
+        <v>28370.02</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>19.571027</v>
+        <v>6.97730121</v>
       </c>
       <c r="E3" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Geopolitics</t>
+          <t>Business/Economy</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>18435.53</v>
+        <v>26854.86</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>7.09241858</v>
+        <v>6.60466391</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Business/Economy</t>
+          <t>Geopolitics</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3303.59</v>
+        <v>12206.22</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1.27093949</v>
+        <v>3.00198849</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sports</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2222.22</v>
+        <v>554.28</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.8549206</v>
+        <v>0.1363192</v>
       </c>
       <c r="E6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Culture</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>487.8</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.11996916</v>
+      </c>
+      <c r="E7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>259932.91</v>
-      </c>
-      <c r="D7" s="6" t="n">
+      <c r="C8" s="5" t="n">
+        <v>406604.49</v>
+      </c>
+      <c r="D8" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="E7" s="4" t="n">
-        <v>259</v>
+      <c r="E8" s="4" t="n">
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -613,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E268"/>
+  <dimension ref="A1:E274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6257,6 +6278,132 @@
         <v>205</v>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Business/Economy</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="n">
+        <v>26854.86</v>
+      </c>
+      <c r="D269" s="3" t="n">
+        <v>6.60466391</v>
+      </c>
+      <c r="E269" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="n">
+        <v>554.28</v>
+      </c>
+      <c r="D270" s="3" t="n">
+        <v>0.1363192</v>
+      </c>
+      <c r="E270" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Culture</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="n">
+        <v>487.8</v>
+      </c>
+      <c r="D271" s="3" t="n">
+        <v>0.11996916</v>
+      </c>
+      <c r="E271" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Geopolitics</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="n">
+        <v>12206.22</v>
+      </c>
+      <c r="D272" s="3" t="n">
+        <v>3.00198849</v>
+      </c>
+      <c r="E272" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Tech &amp; Science</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="n">
+        <v>28370.02</v>
+      </c>
+      <c r="D273" s="3" t="n">
+        <v>6.97730121</v>
+      </c>
+      <c r="E273" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="n">
+        <v>338131.31</v>
+      </c>
+      <c r="D274" s="3" t="n">
+        <v>83.15975802</v>
+      </c>
+      <c r="E274" t="n">
+        <v>216</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>